<commit_message>
Group discount bucket lift by B2B support
Co-authored-by: bhannigan-cpu <bhannigan-cpu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/analysis/member_monday/output/member_monday_case_study.xlsx
+++ b/analysis/member_monday/output/member_monday_case_study.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Class Summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Supplier Summary" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Discount Buckets" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="B2B Bucket Lift" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25939,4 +25940,605 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>discount_bucket</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>b2b_support_segment</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>sku_count</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>active_skus</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>positive_lift_skus</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>positive_lift_sku_rate</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>l10_non_promo_daily_avg</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>member_monday_sales</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>incremental_sales</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>weighted_lift_pct</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>avg_discount_pct</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>weighted_discount_pct</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>weighted_b2b_discount_pct</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>weighted_rec_discount_pct</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>lift_per_discount_point</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>&lt;10%</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>With No B2B Discount</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>206.76</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-206.76</v>
+      </c>
+      <c r="J2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.05023500000000001</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.04952137744244534</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0.04892301184433165</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.4799667101953956</v>
+      </c>
+      <c r="O2" t="n">
+        <v>-20.19329937181611</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>&lt;10%</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>With 5%+ Incremental B2B Discount</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>23</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.08695652173913043</v>
+      </c>
+      <c r="G3" t="n">
+        <v>935.76</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1170.95</v>
+      </c>
+      <c r="I3" t="n">
+        <v>235.1900000000001</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.2513358126015218</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.0543304347826087</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.06075856843635121</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.4362000213730016</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.4980013410683342</v>
+      </c>
+      <c r="O3" t="n">
+        <v>4.136631574274391</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>10-14.9%</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>With No B2B Discount</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>29</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.03448275862068965</v>
+      </c>
+      <c r="G4" t="n">
+        <v>32.25</v>
+      </c>
+      <c r="H4" t="n">
+        <v>220.55</v>
+      </c>
+      <c r="I4" t="n">
+        <v>188.3</v>
+      </c>
+      <c r="J4" t="n">
+        <v>5.838759689922481</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.1137931034482759</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.4343107229500243</v>
+      </c>
+      <c r="O4" t="n">
+        <v>48.65633074935401</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>10-14.9%</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>With 5%+ Incremental B2B Discount</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>65.42</v>
+      </c>
+      <c r="H5" t="n">
+        <v>160.2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>94.78000000000002</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1.448792418220728</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.116</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.4614499082849282</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.3994768266585142</v>
+      </c>
+      <c r="O5" t="n">
+        <v>12.0732701518394</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>15-19.9%</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>With No B2B Discount</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>89</v>
+      </c>
+      <c r="D6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.0898876404494382</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2455.41</v>
+      </c>
+      <c r="H6" t="n">
+        <v>3379.32</v>
+      </c>
+      <c r="I6" t="n">
+        <v>923.9099999999999</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.3762752452747199</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.1621640449438202</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0.160649654029266</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.2356128291586384</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.3881192312402538</v>
+      </c>
+      <c r="O6" t="n">
+        <v>2.342210118959688</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>15-19.9%</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>With 5%+ Incremental B2B Discount</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>68</v>
+      </c>
+      <c r="D7" t="n">
+        <v>18</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.1176470588235294</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1580.47</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1496.78</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-83.6899999999996</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-0.0529526027067895</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.1583794117647059</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0.1623486051617557</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0.45097261827178</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.4563663834175912</v>
+      </c>
+      <c r="O7" t="n">
+        <v>-0.3261660465393607</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>20-24.9%</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>With No B2B Discount</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>20</v>
+      </c>
+      <c r="D8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G8" t="n">
+        <v>49.6</v>
+      </c>
+      <c r="H8" t="n">
+        <v>157.38</v>
+      </c>
+      <c r="I8" t="n">
+        <v>107.78</v>
+      </c>
+      <c r="J8" t="n">
+        <v>2.172983870967742</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.212585</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0.2140357258064516</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0.2145455140798952</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.2892655241935484</v>
+      </c>
+      <c r="O8" t="n">
+        <v>10.15243535993953</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>20-24.9%</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>With 5%+ Incremental B2B Discount</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>52</v>
+      </c>
+      <c r="D9" t="n">
+        <v>9</v>
+      </c>
+      <c r="E9" t="n">
+        <v>7</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.1346153846153846</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3906.22</v>
+      </c>
+      <c r="H9" t="n">
+        <v>4084.41</v>
+      </c>
+      <c r="I9" t="n">
+        <v>178.1899999999996</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.04561699033848569</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.217273076923077</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0.2195779551586956</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0.2736969149203066</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.4194381340528695</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.2077484978194506</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>25%+</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>With No B2B Discount</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>52</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.0576923076923077</v>
+      </c>
+      <c r="G10" t="n">
+        <v>161.32</v>
+      </c>
+      <c r="H10" t="n">
+        <v>223.15</v>
+      </c>
+      <c r="I10" t="n">
+        <v>61.82999999999998</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.3832754773121744</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0.2821384615384616</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0.292459831391024</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0.3430665760869565</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.4882382501145212</v>
+      </c>
+      <c r="O10" t="n">
+        <v>1.310523484504538</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>25%+</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>With 5%+ Incremental B2B Discount</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>9</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.1111111111111111</v>
+      </c>
+      <c r="G11" t="n">
+        <v>178.8</v>
+      </c>
+      <c r="H11" t="n">
+        <v>223.87</v>
+      </c>
+      <c r="I11" t="n">
+        <v>45.07000000000002</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.2520693512304252</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0.2722222222222223</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0.4888053691275168</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.4999502460850112</v>
+      </c>
+      <c r="O11" t="n">
+        <v>1.008277404921701</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Use class sales bars for lift chart
Co-authored-by: bhannigan-cpu <bhannigan-cpu@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/analysis/member_monday/output/member_monday_case_study.xlsx
+++ b/analysis/member_monday/output/member_monday_case_study.xlsx
@@ -12,7 +12,6 @@
     <sheet name="Class Summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Supplier Summary" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Discount Buckets" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="B2B Bucket Lift" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25940,605 +25939,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:O11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>discount_bucket</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>b2b_support_segment</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>sku_count</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>active_skus</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>positive_lift_skus</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>positive_lift_sku_rate</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>l10_non_promo_daily_avg</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>member_monday_sales</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>incremental_sales</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>weighted_lift_pct</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>avg_discount_pct</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>weighted_discount_pct</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>weighted_b2b_discount_pct</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>weighted_rec_discount_pct</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>lift_per_discount_point</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>&lt;10%</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>With No B2B Discount</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>20</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>206.76</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>-206.76</v>
-      </c>
-      <c r="J2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.05023500000000001</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.04952137744244534</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.04892301184433165</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.4799667101953956</v>
-      </c>
-      <c r="O2" t="n">
-        <v>-20.19329937181611</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>&lt;10%</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>With 5%+ Incremental B2B Discount</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>23</v>
-      </c>
-      <c r="D3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.08695652173913043</v>
-      </c>
-      <c r="G3" t="n">
-        <v>935.76</v>
-      </c>
-      <c r="H3" t="n">
-        <v>1170.95</v>
-      </c>
-      <c r="I3" t="n">
-        <v>235.1900000000001</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.2513358126015218</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.0543304347826087</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.06075856843635121</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.4362000213730016</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.4980013410683342</v>
-      </c>
-      <c r="O3" t="n">
-        <v>4.136631574274391</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>10-14.9%</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>With No B2B Discount</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>29</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.03448275862068965</v>
-      </c>
-      <c r="G4" t="n">
-        <v>32.25</v>
-      </c>
-      <c r="H4" t="n">
-        <v>220.55</v>
-      </c>
-      <c r="I4" t="n">
-        <v>188.3</v>
-      </c>
-      <c r="J4" t="n">
-        <v>5.838759689922481</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0.1137931034482759</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0.4343107229500243</v>
-      </c>
-      <c r="O4" t="n">
-        <v>48.65633074935401</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>10-14.9%</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>With 5%+ Incremental B2B Discount</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>10</v>
-      </c>
-      <c r="D5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G5" t="n">
-        <v>65.42</v>
-      </c>
-      <c r="H5" t="n">
-        <v>160.2</v>
-      </c>
-      <c r="I5" t="n">
-        <v>94.78000000000002</v>
-      </c>
-      <c r="J5" t="n">
-        <v>1.448792418220728</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.4614499082849282</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.3994768266585142</v>
-      </c>
-      <c r="O5" t="n">
-        <v>12.0732701518394</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>15-19.9%</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>With No B2B Discount</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>89</v>
-      </c>
-      <c r="D6" t="n">
-        <v>10</v>
-      </c>
-      <c r="E6" t="n">
-        <v>8</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.0898876404494382</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2455.41</v>
-      </c>
-      <c r="H6" t="n">
-        <v>3379.32</v>
-      </c>
-      <c r="I6" t="n">
-        <v>923.9099999999999</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0.3762752452747199</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.1621640449438202</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.160649654029266</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0.2356128291586384</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0.3881192312402538</v>
-      </c>
-      <c r="O6" t="n">
-        <v>2.342210118959688</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>15-19.9%</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>With 5%+ Incremental B2B Discount</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>68</v>
-      </c>
-      <c r="D7" t="n">
-        <v>18</v>
-      </c>
-      <c r="E7" t="n">
-        <v>8</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.1176470588235294</v>
-      </c>
-      <c r="G7" t="n">
-        <v>1580.47</v>
-      </c>
-      <c r="H7" t="n">
-        <v>1496.78</v>
-      </c>
-      <c r="I7" t="n">
-        <v>-83.6899999999996</v>
-      </c>
-      <c r="J7" t="n">
-        <v>-0.0529526027067895</v>
-      </c>
-      <c r="K7" t="n">
-        <v>0.1583794117647059</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.1623486051617557</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0.45097261827178</v>
-      </c>
-      <c r="N7" t="n">
-        <v>0.4563663834175912</v>
-      </c>
-      <c r="O7" t="n">
-        <v>-0.3261660465393607</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>20-24.9%</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>With No B2B Discount</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>20</v>
-      </c>
-      <c r="D8" t="n">
-        <v>3</v>
-      </c>
-      <c r="E8" t="n">
-        <v>3</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="G8" t="n">
-        <v>49.6</v>
-      </c>
-      <c r="H8" t="n">
-        <v>157.38</v>
-      </c>
-      <c r="I8" t="n">
-        <v>107.78</v>
-      </c>
-      <c r="J8" t="n">
-        <v>2.172983870967742</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0.212585</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.2140357258064516</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.2145455140798952</v>
-      </c>
-      <c r="N8" t="n">
-        <v>0.2892655241935484</v>
-      </c>
-      <c r="O8" t="n">
-        <v>10.15243535993953</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>20-24.9%</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>With 5%+ Incremental B2B Discount</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>52</v>
-      </c>
-      <c r="D9" t="n">
-        <v>9</v>
-      </c>
-      <c r="E9" t="n">
-        <v>7</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0.1346153846153846</v>
-      </c>
-      <c r="G9" t="n">
-        <v>3906.22</v>
-      </c>
-      <c r="H9" t="n">
-        <v>4084.41</v>
-      </c>
-      <c r="I9" t="n">
-        <v>178.1899999999996</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0.04561699033848569</v>
-      </c>
-      <c r="K9" t="n">
-        <v>0.217273076923077</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0.2195779551586956</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0.2736969149203066</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0.4194381340528695</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0.2077484978194506</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>25%+</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>With No B2B Discount</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>52</v>
-      </c>
-      <c r="D10" t="n">
-        <v>3</v>
-      </c>
-      <c r="E10" t="n">
-        <v>3</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0.0576923076923077</v>
-      </c>
-      <c r="G10" t="n">
-        <v>161.32</v>
-      </c>
-      <c r="H10" t="n">
-        <v>223.15</v>
-      </c>
-      <c r="I10" t="n">
-        <v>61.82999999999998</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.3832754773121744</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0.2821384615384616</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.292459831391024</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0.3430665760869565</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0.4882382501145212</v>
-      </c>
-      <c r="O10" t="n">
-        <v>1.310523484504538</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>25%+</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>With 5%+ Incremental B2B Discount</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>9</v>
-      </c>
-      <c r="D11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" t="n">
-        <v>0.1111111111111111</v>
-      </c>
-      <c r="G11" t="n">
-        <v>178.8</v>
-      </c>
-      <c r="H11" t="n">
-        <v>223.87</v>
-      </c>
-      <c r="I11" t="n">
-        <v>45.07000000000002</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0.2520693512304252</v>
-      </c>
-      <c r="K11" t="n">
-        <v>0.2722222222222223</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0.4888053691275168</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0.4999502460850112</v>
-      </c>
-      <c r="O11" t="n">
-        <v>1.008277404921701</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>